<commit_message>
qPCR macro 3.4: fix compilacion Call OrdenarMuestras y hojas Datos/Calculos con formulas
- Corrige error de sintaxis: Call OrdenarMuestras(orden) (requerido en VBA con Call)
- Nueva hoja Datos: tabla muestra x gen leida del RAW
- Nueva hoja Calculos: formulas SUMIFS/AVERAGEIFS para dCt y promedio C
- Resultados enlaza a Calculos (ddCt y 2^(-ddCt) con formulas Excel)
- Plantilla y DESCARGA.md actualizados

Co-authored-by: carlosvibecoding <carlosvibecoding@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/qPCR_plantilla.xlsx
+++ b/qPCR_plantilla.xlsx
@@ -11,6 +11,8 @@
     <sheet name="RAW" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Resultados" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="GLOBAL" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Datos" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Calculos" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -39,6 +41,9 @@
     <font>
       <color rgb="000070C0"/>
       <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -61,11 +66,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -431,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A18"/>
+  <dimension ref="A1:A20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="95" customWidth="1" min="1" max="1"/>
@@ -498,50 +504,64 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Resultados — datos y cálculos (bloque PPIA a la izquierda, SYP a la derecha)</t>
+          <t xml:space="preserve">  • Datos — tabla leída del RAW (Ct por muestra y gen)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • GLOBAL — resumen por sujeto (controles | suicidas)</t>
+          <t xml:space="preserve">  • Calculos — ΔCt y promedio C con fórmulas Excel (auditable)</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr"/>
+      <c r="A13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Resultados — presentación (fórmulas enlazadas a Calculos)</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Cálculos (por cada gen control PPIA y SYP):</t>
+          <t xml:space="preserve">  • GLOBAL — resumen por sujeto (controles | suicidas)</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Paso 1: ΔCt = Ct mean (gen problema) − Ct mean (control)</t>
-        </is>
-      </c>
+      <c r="A15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Paso 2: Promedio del paso 1 solo en muestras C (C1, C12, …)</t>
+          <t>Cálculos (por cada gen control PPIA y SYP):</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Paso 3: ΔΔCt = ΔCt − promedio del paso 2 (fijo para todas las muestras)</t>
+          <t xml:space="preserve">  Paso 1: ΔCt = Ct mean (gen problema) − Ct mean (control)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Paso 2: Promedio del paso 1 solo en muestras C (C1, C12, …)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Paso 3: ΔΔCt = ΔCt − promedio del paso 2 (fijo para todas las muestras)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
         <is>
           <t xml:space="preserve">  Paso 4: 2^(−ΔΔCt)</t>
         </is>
@@ -618,4 +638,116 @@
   <sheetData/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Muestra</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Gen</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Ct 1</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Ct 2</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Ct Mean</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Ct SD</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>Indet</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Muestra</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Ct GOI</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Ct PPIA</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Ct SYP</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>dCt PPIA</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>dCt SYP</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>Gen interes</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>Prom dCt (C) PPIA</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>Prom dCt (C) SYP</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
qPCR macro 3.8: grupos configurables y botones decorados en RAW
- Muestras: cualquier prefijo letras+numero (C10, S5, A12, ALC3)
- Instrucciones B21/B22: prefijos control y nombres de grupo
- GLOBAL: tabla por prefijo con etiqueta configurable
- Botones redondeados a la derecha (columna N), pegado desde A3
- Python: mismo criterio de grupos en processor/plantilla

Co-authored-by: carlosvibecoding <carlosvibecoding@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/qPCR_plantilla.xlsx
+++ b/qPCR_plantilla.xlsx
@@ -22,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -33,6 +33,15 @@
     <font>
       <b val="1"/>
       <sz val="14"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="0000468C"/>
+      <sz val="11"/>
     </font>
     <font>
       <i val="1"/>
@@ -66,12 +75,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -437,10 +448,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A20"/>
+  <dimension ref="A1:B26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="95" customWidth="1" min="1" max="1"/>
+    <col width="55" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -525,7 +537,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • GLOBAL — resumen por sujeto (controles | suicidas)</t>
+          <t xml:space="preserve">  • GLOBAL — resumen por grupo (controles + cada prefijo de muestra)</t>
         </is>
       </c>
     </row>
@@ -535,33 +547,81 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Cálculos (por cada gen control PPIA y SYP):</t>
+          <t>CONFIGURACIÓN DE GRUPOS (editable):</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Paso 1: ΔCt = Ct mean (gen problema) − Ct mean (control)</t>
+          <t xml:space="preserve">  B21 — Prefijos control para promedio ΔCt (ej: C   o   C,CTRL)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Paso 2: Promedio del paso 1 solo en muestras C (C1, C12, …)</t>
+          <t xml:space="preserve">  B22 — Nombres de grupos (ej: C=Controles;S=Suicidas;A=Alcohólicos)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
+          <t xml:space="preserve">  Si B22 está vacío, se usan nombres automáticos según el prefijo (C, S, A…).</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>CONFIGURACIÓN DE GRUPOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Prefijos control (promedio ΔCt):</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Nombres grupos (C=Controles;S=Suicidas;A=Alcohólicos):</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Paso 1: ΔCt = Ct mean (gen problema) − Ct mean (control)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Paso 2: Promedio del paso 1 solo en muestras control (prefijo B21)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
           <t xml:space="preserve">  Paso 3: ΔΔCt = ΔCt − promedio del paso 2 (fijo para todas las muestras)</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
+    <row r="26">
+      <c r="A26" t="inlineStr">
         <is>
           <t xml:space="preserve">  Paso 4: 2^(−ΔΔCt)</t>
         </is>
@@ -578,7 +638,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N1"/>
+  <dimension ref="A1:N3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -598,14 +658,21 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
-        <is>
-          <t>Pegue aquí el export del termociclador (Sample Name, Target Name, Ct, Ct Mean, Ct SD…)</t>
-        </is>
-      </c>
-      <c r="N1" s="3" t="inlineStr">
-        <is>
-          <t>← Importe Modulo_qPCR.bas y asigne la macro ProcesarPlaca a un botón aquí</t>
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>qPCR — Pegar export StepOne desde fila 3 (celda A3)</t>
+        </is>
+      </c>
+      <c r="N1" s="4" t="inlineStr">
+        <is>
+          <t>Botones → (se crean al abrir el libro con la macro importada)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Pegue aquí el export (Sample Name, Target Name, Ct, Ct Mean, Ct SD…)</t>
         </is>
       </c>
     </row>
@@ -650,37 +717,37 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="6" t="inlineStr">
         <is>
           <t>Muestra</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
+      <c r="B1" s="6" t="inlineStr">
         <is>
           <t>Gen</t>
         </is>
       </c>
-      <c r="C1" s="4" t="inlineStr">
+      <c r="C1" s="6" t="inlineStr">
         <is>
           <t>Ct 1</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="D1" s="6" t="inlineStr">
         <is>
           <t>Ct 2</t>
         </is>
       </c>
-      <c r="E1" s="4" t="inlineStr">
+      <c r="E1" s="6" t="inlineStr">
         <is>
           <t>Ct Mean</t>
         </is>
       </c>
-      <c r="F1" s="4" t="inlineStr">
+      <c r="F1" s="6" t="inlineStr">
         <is>
           <t>Ct SD</t>
         </is>
       </c>
-      <c r="G1" s="4" t="inlineStr">
+      <c r="G1" s="6" t="inlineStr">
         <is>
           <t>Indet</t>
         </is>
@@ -701,47 +768,47 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="6" t="inlineStr">
         <is>
           <t>Muestra</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
+      <c r="B1" s="6" t="inlineStr">
         <is>
           <t>Ct GOI</t>
         </is>
       </c>
-      <c r="C1" s="4" t="inlineStr">
+      <c r="C1" s="6" t="inlineStr">
         <is>
           <t>Ct PPIA</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="D1" s="6" t="inlineStr">
         <is>
           <t>Ct SYP</t>
         </is>
       </c>
-      <c r="E1" s="4" t="inlineStr">
+      <c r="E1" s="6" t="inlineStr">
         <is>
           <t>dCt PPIA</t>
         </is>
       </c>
-      <c r="F1" s="4" t="inlineStr">
+      <c r="F1" s="6" t="inlineStr">
         <is>
           <t>dCt SYP</t>
         </is>
       </c>
-      <c r="G1" s="4" t="inlineStr">
+      <c r="G1" s="6" t="inlineStr">
         <is>
           <t>Gen interes</t>
         </is>
       </c>
-      <c r="H1" s="4" t="inlineStr">
+      <c r="H1" s="6" t="inlineStr">
         <is>
           <t>Prom dCt (C) PPIA</t>
         </is>
       </c>
-      <c r="I1" s="4" t="inlineStr">
+      <c r="I1" s="6" t="inlineStr">
         <is>
           <t>Prom dCt (C) SYP</t>
         </is>

</xml_diff>

<commit_message>
qPCR 3.9: panel RAW izquierda, texto ASCII, logo opcional (ElegirLogo)
Co-authored-by: carlosvibecoding <carlosvibecoding@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/qPCR_plantilla.xlsx
+++ b/qPCR_plantilla.xlsx
@@ -22,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -39,11 +39,6 @@
       <sz val="12"/>
     </font>
     <font>
-      <b val="1"/>
-      <color rgb="0000468C"/>
-      <sz val="11"/>
-    </font>
-    <font>
       <i val="1"/>
       <color rgb="00666666"/>
     </font>
@@ -55,12 +50,17 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EDF2F7"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -79,10 +79,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B26"/>
+  <dimension ref="A1:B27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="95" customWidth="1" min="1" max="1"/>
@@ -602,26 +602,34 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Paso 1: ΔCt = Ct mean (gen problema) − Ct mean (control)</t>
+          <t>Logo (opcional):</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Paso 2: Promedio del paso 1 solo en muestras control (prefijo B21)</t>
-        </is>
-      </c>
+          <t>Ruta imagen o figura qPCR_logo en esta hoja (macro ElegirLogo):</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Paso 3: ΔΔCt = ΔCt − promedio del paso 2 (fijo para todas las muestras)</t>
+          <t xml:space="preserve">  Paso 2: Promedio del paso 1 solo en muestras control (prefijo B21)</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Paso 3: ΔΔCt = ΔCt − promedio del paso 2 (fijo para todas las muestras)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
         <is>
           <t xml:space="preserve">  Paso 4: 2^(−ΔΔCt)</t>
         </is>
@@ -638,7 +646,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N3"/>
+  <dimension ref="A1:K3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -658,21 +666,29 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
-        <is>
-          <t>qPCR — Pegar export StepOne desde fila 3 (celda A3)</t>
-        </is>
-      </c>
-      <c r="N1" s="4" t="inlineStr">
-        <is>
-          <t>Botones → (se crean al abrir el libro con la macro importada)</t>
-        </is>
-      </c>
+      <c r="A1" s="3" t="inlineStr"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>(Botones e imagen: macro InstalarBotones / ElegirLogo al abrir el .xlsm)</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="n"/>
+      <c r="C2" s="3" t="n"/>
+      <c r="D2" s="3" t="n"/>
+      <c r="E2" s="3" t="n"/>
+      <c r="F2" s="3" t="n"/>
+      <c r="G2" s="3" t="n"/>
+      <c r="H2" s="3" t="n"/>
+      <c r="I2" s="3" t="n"/>
+      <c r="J2" s="3" t="n"/>
+      <c r="K2" s="3" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>Pegue aquí el export (Sample Name, Target Name, Ct, Ct Mean, Ct SD…)</t>
+          <t>Pegue aqui el export StepOne (Sample Name, Target Name, Ct, Ct Mean, Ct SD...)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
qPCR 4.0: boton fijo con imagen de raton embebida en plantilla
- Imagen raton_procesar.png en qpcr/assets y hoja oculta Recursos
- Clic en raton ejecuta ProcesarPlaca; panel izquierda sin ElegirLogo
- Sin caracteres especiales en celdas (evita texto roto en Excel online)

Co-authored-by: carlosvibecoding <carlosvibecoding@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/qPCR_plantilla.xlsx
+++ b/qPCR_plantilla.xlsx
@@ -22,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -41,10 +41,6 @@
     <font>
       <i val="1"/>
       <color rgb="00666666"/>
-    </font>
-    <font>
-      <color rgb="000070C0"/>
-      <sz val="9"/>
     </font>
     <font>
       <b val="1"/>
@@ -75,14 +71,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -669,11 +664,7 @@
       <c r="A1" s="3" t="inlineStr"/>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>(Botones e imagen: macro InstalarBotones / ElegirLogo al abrir el .xlsm)</t>
-        </is>
-      </c>
+      <c r="A2" s="3" t="inlineStr"/>
       <c r="B2" s="3" t="n"/>
       <c r="C2" s="3" t="n"/>
       <c r="D2" s="3" t="n"/>
@@ -686,7 +677,7 @@
       <c r="K2" s="3" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>Pegue aqui el export StepOne (Sample Name, Target Name, Ct, Ct Mean, Ct SD...)</t>
         </is>
@@ -733,37 +724,37 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="6" t="inlineStr">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>Muestra</t>
         </is>
       </c>
-      <c r="B1" s="6" t="inlineStr">
+      <c r="B1" s="5" t="inlineStr">
         <is>
           <t>Gen</t>
         </is>
       </c>
-      <c r="C1" s="6" t="inlineStr">
+      <c r="C1" s="5" t="inlineStr">
         <is>
           <t>Ct 1</t>
         </is>
       </c>
-      <c r="D1" s="6" t="inlineStr">
+      <c r="D1" s="5" t="inlineStr">
         <is>
           <t>Ct 2</t>
         </is>
       </c>
-      <c r="E1" s="6" t="inlineStr">
+      <c r="E1" s="5" t="inlineStr">
         <is>
           <t>Ct Mean</t>
         </is>
       </c>
-      <c r="F1" s="6" t="inlineStr">
+      <c r="F1" s="5" t="inlineStr">
         <is>
           <t>Ct SD</t>
         </is>
       </c>
-      <c r="G1" s="6" t="inlineStr">
+      <c r="G1" s="5" t="inlineStr">
         <is>
           <t>Indet</t>
         </is>
@@ -784,47 +775,47 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="6" t="inlineStr">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>Muestra</t>
         </is>
       </c>
-      <c r="B1" s="6" t="inlineStr">
+      <c r="B1" s="5" t="inlineStr">
         <is>
           <t>Ct GOI</t>
         </is>
       </c>
-      <c r="C1" s="6" t="inlineStr">
+      <c r="C1" s="5" t="inlineStr">
         <is>
           <t>Ct PPIA</t>
         </is>
       </c>
-      <c r="D1" s="6" t="inlineStr">
+      <c r="D1" s="5" t="inlineStr">
         <is>
           <t>Ct SYP</t>
         </is>
       </c>
-      <c r="E1" s="6" t="inlineStr">
+      <c r="E1" s="5" t="inlineStr">
         <is>
           <t>dCt PPIA</t>
         </is>
       </c>
-      <c r="F1" s="6" t="inlineStr">
+      <c r="F1" s="5" t="inlineStr">
         <is>
           <t>dCt SYP</t>
         </is>
       </c>
-      <c r="G1" s="6" t="inlineStr">
+      <c r="G1" s="5" t="inlineStr">
         <is>
           <t>Gen interes</t>
         </is>
       </c>
-      <c r="H1" s="6" t="inlineStr">
+      <c r="H1" s="5" t="inlineStr">
         <is>
           <t>Prom dCt (C) PPIA</t>
         </is>
       </c>
-      <c r="I1" s="6" t="inlineStr">
+      <c r="I1" s="5" t="inlineStr">
         <is>
           <t>Prom dCt (C) SYP</t>
         </is>

</xml_diff>

<commit_message>
qPCR 4.1: raton lab mono, fondo ADN molecular, tema laboratorio
- Assets: raton_boton.png, fondo_cabecera_raw.png (generados y optimizados)
- RAW: paleta lab, cabecera con watermark ADN, boton raton fijo
- Macro InstalarBotones: fondo + raton desde hoja Recursos

Co-authored-by: carlosvibecoding <carlosvibecoding@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/qPCR_plantilla.xlsx
+++ b/qPCR_plantilla.xlsx
@@ -13,6 +13,7 @@
     <sheet name="GLOBAL" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Datos" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Calculos" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Recursos" sheetId="7" state="hidden" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -40,13 +41,14 @@
     </font>
     <font>
       <i val="1"/>
-      <color rgb="00666666"/>
+      <color rgb="0037474F"/>
+      <sz val="10"/>
     </font>
     <font>
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -55,7 +57,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EDF2F7"/>
+        <fgColor rgb="00E0F2F1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F0F7FA"/>
       </patternFill>
     </fill>
   </fills>
@@ -71,12 +78,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -152,6 +160,61 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="685800" cy="685800"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6858000" cy="914400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -463,7 +526,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1. Pegue el export del termociclador (StepOne) en la hoja RAW, desde la celda A1.</t>
+          <t>1. Pegue el export del termociclador (StepOne) en la hoja RAW, desde la celda A3.</t>
         </is>
       </c>
     </row>
@@ -597,17 +660,21 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Logo (opcional):</t>
+          <t>Boton procesar:</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Clic en el raton de la hoja RAW = Procesar placa (macro 4.1)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Ruta imagen o figura qPCR_logo en esta hoja (macro ElegirLogo):</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr"/>
+          <t xml:space="preserve">  Paso 1: ΔCt = Ct mean (gen problema) − Ct mean (control)</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -641,7 +708,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:Q79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -658,13 +725,30 @@
     <col width="12" customWidth="1" min="12" max="12"/>
     <col width="12" customWidth="1" min="13" max="13"/>
     <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="3" t="inlineStr"/>
-    </row>
-    <row r="2">
-      <c r="A2" s="3" t="inlineStr"/>
+    <row r="1" ht="8" customHeight="1">
+      <c r="A1" s="3" t="n"/>
+      <c r="B1" s="3" t="n"/>
+      <c r="C1" s="3" t="n"/>
+      <c r="D1" s="3" t="n"/>
+      <c r="E1" s="3" t="n"/>
+      <c r="F1" s="3" t="n"/>
+      <c r="G1" s="3" t="n"/>
+      <c r="H1" s="3" t="n"/>
+      <c r="I1" s="3" t="n"/>
+      <c r="J1" s="3" t="n"/>
+      <c r="K1" s="3" t="n"/>
+      <c r="L1" s="3" t="n"/>
+      <c r="M1" s="3" t="n"/>
+      <c r="N1" s="3" t="n"/>
+      <c r="O1" s="3" t="n"/>
+      <c r="P1" s="3" t="n"/>
+      <c r="Q1" s="3" t="n"/>
+    </row>
+    <row r="2" ht="52" customHeight="1">
+      <c r="A2" s="3" t="n"/>
       <c r="B2" s="3" t="n"/>
       <c r="C2" s="3" t="n"/>
       <c r="D2" s="3" t="n"/>
@@ -675,6 +759,12 @@
       <c r="I2" s="3" t="n"/>
       <c r="J2" s="3" t="n"/>
       <c r="K2" s="3" t="n"/>
+      <c r="L2" s="3" t="n"/>
+      <c r="M2" s="3" t="n"/>
+      <c r="N2" s="3" t="n"/>
+      <c r="O2" s="3" t="n"/>
+      <c r="P2" s="3" t="n"/>
+      <c r="Q2" s="3" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
@@ -682,6 +772,1466 @@
           <t>Pegue aqui el export StepOne (Sample Name, Target Name, Ct, Ct Mean, Ct SD...)</t>
         </is>
       </c>
+      <c r="B3" s="5" t="n"/>
+      <c r="C3" s="5" t="n"/>
+      <c r="D3" s="5" t="n"/>
+      <c r="E3" s="5" t="n"/>
+      <c r="F3" s="5" t="n"/>
+      <c r="G3" s="5" t="n"/>
+      <c r="H3" s="5" t="n"/>
+      <c r="I3" s="5" t="n"/>
+      <c r="J3" s="5" t="n"/>
+      <c r="K3" s="5" t="n"/>
+      <c r="L3" s="5" t="n"/>
+      <c r="M3" s="5" t="n"/>
+      <c r="N3" s="5" t="n"/>
+      <c r="O3" s="5" t="n"/>
+      <c r="P3" s="5" t="n"/>
+      <c r="Q3" s="5" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="n"/>
+      <c r="B4" s="5" t="n"/>
+      <c r="C4" s="5" t="n"/>
+      <c r="D4" s="5" t="n"/>
+      <c r="E4" s="5" t="n"/>
+      <c r="F4" s="5" t="n"/>
+      <c r="G4" s="5" t="n"/>
+      <c r="H4" s="5" t="n"/>
+      <c r="I4" s="5" t="n"/>
+      <c r="J4" s="5" t="n"/>
+      <c r="K4" s="5" t="n"/>
+      <c r="L4" s="5" t="n"/>
+      <c r="M4" s="5" t="n"/>
+      <c r="N4" s="5" t="n"/>
+      <c r="O4" s="5" t="n"/>
+      <c r="P4" s="5" t="n"/>
+      <c r="Q4" s="5" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="n"/>
+      <c r="B5" s="5" t="n"/>
+      <c r="C5" s="5" t="n"/>
+      <c r="D5" s="5" t="n"/>
+      <c r="E5" s="5" t="n"/>
+      <c r="F5" s="5" t="n"/>
+      <c r="G5" s="5" t="n"/>
+      <c r="H5" s="5" t="n"/>
+      <c r="I5" s="5" t="n"/>
+      <c r="J5" s="5" t="n"/>
+      <c r="K5" s="5" t="n"/>
+      <c r="L5" s="5" t="n"/>
+      <c r="M5" s="5" t="n"/>
+      <c r="N5" s="5" t="n"/>
+      <c r="O5" s="5" t="n"/>
+      <c r="P5" s="5" t="n"/>
+      <c r="Q5" s="5" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="n"/>
+      <c r="B6" s="5" t="n"/>
+      <c r="C6" s="5" t="n"/>
+      <c r="D6" s="5" t="n"/>
+      <c r="E6" s="5" t="n"/>
+      <c r="F6" s="5" t="n"/>
+      <c r="G6" s="5" t="n"/>
+      <c r="H6" s="5" t="n"/>
+      <c r="I6" s="5" t="n"/>
+      <c r="J6" s="5" t="n"/>
+      <c r="K6" s="5" t="n"/>
+      <c r="L6" s="5" t="n"/>
+      <c r="M6" s="5" t="n"/>
+      <c r="N6" s="5" t="n"/>
+      <c r="O6" s="5" t="n"/>
+      <c r="P6" s="5" t="n"/>
+      <c r="Q6" s="5" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="n"/>
+      <c r="B7" s="5" t="n"/>
+      <c r="C7" s="5" t="n"/>
+      <c r="D7" s="5" t="n"/>
+      <c r="E7" s="5" t="n"/>
+      <c r="F7" s="5" t="n"/>
+      <c r="G7" s="5" t="n"/>
+      <c r="H7" s="5" t="n"/>
+      <c r="I7" s="5" t="n"/>
+      <c r="J7" s="5" t="n"/>
+      <c r="K7" s="5" t="n"/>
+      <c r="L7" s="5" t="n"/>
+      <c r="M7" s="5" t="n"/>
+      <c r="N7" s="5" t="n"/>
+      <c r="O7" s="5" t="n"/>
+      <c r="P7" s="5" t="n"/>
+      <c r="Q7" s="5" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="n"/>
+      <c r="B8" s="5" t="n"/>
+      <c r="C8" s="5" t="n"/>
+      <c r="D8" s="5" t="n"/>
+      <c r="E8" s="5" t="n"/>
+      <c r="F8" s="5" t="n"/>
+      <c r="G8" s="5" t="n"/>
+      <c r="H8" s="5" t="n"/>
+      <c r="I8" s="5" t="n"/>
+      <c r="J8" s="5" t="n"/>
+      <c r="K8" s="5" t="n"/>
+      <c r="L8" s="5" t="n"/>
+      <c r="M8" s="5" t="n"/>
+      <c r="N8" s="5" t="n"/>
+      <c r="O8" s="5" t="n"/>
+      <c r="P8" s="5" t="n"/>
+      <c r="Q8" s="5" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="n"/>
+      <c r="B9" s="5" t="n"/>
+      <c r="C9" s="5" t="n"/>
+      <c r="D9" s="5" t="n"/>
+      <c r="E9" s="5" t="n"/>
+      <c r="F9" s="5" t="n"/>
+      <c r="G9" s="5" t="n"/>
+      <c r="H9" s="5" t="n"/>
+      <c r="I9" s="5" t="n"/>
+      <c r="J9" s="5" t="n"/>
+      <c r="K9" s="5" t="n"/>
+      <c r="L9" s="5" t="n"/>
+      <c r="M9" s="5" t="n"/>
+      <c r="N9" s="5" t="n"/>
+      <c r="O9" s="5" t="n"/>
+      <c r="P9" s="5" t="n"/>
+      <c r="Q9" s="5" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="n"/>
+      <c r="B10" s="5" t="n"/>
+      <c r="C10" s="5" t="n"/>
+      <c r="D10" s="5" t="n"/>
+      <c r="E10" s="5" t="n"/>
+      <c r="F10" s="5" t="n"/>
+      <c r="G10" s="5" t="n"/>
+      <c r="H10" s="5" t="n"/>
+      <c r="I10" s="5" t="n"/>
+      <c r="J10" s="5" t="n"/>
+      <c r="K10" s="5" t="n"/>
+      <c r="L10" s="5" t="n"/>
+      <c r="M10" s="5" t="n"/>
+      <c r="N10" s="5" t="n"/>
+      <c r="O10" s="5" t="n"/>
+      <c r="P10" s="5" t="n"/>
+      <c r="Q10" s="5" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="n"/>
+      <c r="B11" s="5" t="n"/>
+      <c r="C11" s="5" t="n"/>
+      <c r="D11" s="5" t="n"/>
+      <c r="E11" s="5" t="n"/>
+      <c r="F11" s="5" t="n"/>
+      <c r="G11" s="5" t="n"/>
+      <c r="H11" s="5" t="n"/>
+      <c r="I11" s="5" t="n"/>
+      <c r="J11" s="5" t="n"/>
+      <c r="K11" s="5" t="n"/>
+      <c r="L11" s="5" t="n"/>
+      <c r="M11" s="5" t="n"/>
+      <c r="N11" s="5" t="n"/>
+      <c r="O11" s="5" t="n"/>
+      <c r="P11" s="5" t="n"/>
+      <c r="Q11" s="5" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="n"/>
+      <c r="B12" s="5" t="n"/>
+      <c r="C12" s="5" t="n"/>
+      <c r="D12" s="5" t="n"/>
+      <c r="E12" s="5" t="n"/>
+      <c r="F12" s="5" t="n"/>
+      <c r="G12" s="5" t="n"/>
+      <c r="H12" s="5" t="n"/>
+      <c r="I12" s="5" t="n"/>
+      <c r="J12" s="5" t="n"/>
+      <c r="K12" s="5" t="n"/>
+      <c r="L12" s="5" t="n"/>
+      <c r="M12" s="5" t="n"/>
+      <c r="N12" s="5" t="n"/>
+      <c r="O12" s="5" t="n"/>
+      <c r="P12" s="5" t="n"/>
+      <c r="Q12" s="5" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="n"/>
+      <c r="B13" s="5" t="n"/>
+      <c r="C13" s="5" t="n"/>
+      <c r="D13" s="5" t="n"/>
+      <c r="E13" s="5" t="n"/>
+      <c r="F13" s="5" t="n"/>
+      <c r="G13" s="5" t="n"/>
+      <c r="H13" s="5" t="n"/>
+      <c r="I13" s="5" t="n"/>
+      <c r="J13" s="5" t="n"/>
+      <c r="K13" s="5" t="n"/>
+      <c r="L13" s="5" t="n"/>
+      <c r="M13" s="5" t="n"/>
+      <c r="N13" s="5" t="n"/>
+      <c r="O13" s="5" t="n"/>
+      <c r="P13" s="5" t="n"/>
+      <c r="Q13" s="5" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="n"/>
+      <c r="B14" s="5" t="n"/>
+      <c r="C14" s="5" t="n"/>
+      <c r="D14" s="5" t="n"/>
+      <c r="E14" s="5" t="n"/>
+      <c r="F14" s="5" t="n"/>
+      <c r="G14" s="5" t="n"/>
+      <c r="H14" s="5" t="n"/>
+      <c r="I14" s="5" t="n"/>
+      <c r="J14" s="5" t="n"/>
+      <c r="K14" s="5" t="n"/>
+      <c r="L14" s="5" t="n"/>
+      <c r="M14" s="5" t="n"/>
+      <c r="N14" s="5" t="n"/>
+      <c r="O14" s="5" t="n"/>
+      <c r="P14" s="5" t="n"/>
+      <c r="Q14" s="5" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="n"/>
+      <c r="B15" s="5" t="n"/>
+      <c r="C15" s="5" t="n"/>
+      <c r="D15" s="5" t="n"/>
+      <c r="E15" s="5" t="n"/>
+      <c r="F15" s="5" t="n"/>
+      <c r="G15" s="5" t="n"/>
+      <c r="H15" s="5" t="n"/>
+      <c r="I15" s="5" t="n"/>
+      <c r="J15" s="5" t="n"/>
+      <c r="K15" s="5" t="n"/>
+      <c r="L15" s="5" t="n"/>
+      <c r="M15" s="5" t="n"/>
+      <c r="N15" s="5" t="n"/>
+      <c r="O15" s="5" t="n"/>
+      <c r="P15" s="5" t="n"/>
+      <c r="Q15" s="5" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="n"/>
+      <c r="B16" s="5" t="n"/>
+      <c r="C16" s="5" t="n"/>
+      <c r="D16" s="5" t="n"/>
+      <c r="E16" s="5" t="n"/>
+      <c r="F16" s="5" t="n"/>
+      <c r="G16" s="5" t="n"/>
+      <c r="H16" s="5" t="n"/>
+      <c r="I16" s="5" t="n"/>
+      <c r="J16" s="5" t="n"/>
+      <c r="K16" s="5" t="n"/>
+      <c r="L16" s="5" t="n"/>
+      <c r="M16" s="5" t="n"/>
+      <c r="N16" s="5" t="n"/>
+      <c r="O16" s="5" t="n"/>
+      <c r="P16" s="5" t="n"/>
+      <c r="Q16" s="5" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="n"/>
+      <c r="B17" s="5" t="n"/>
+      <c r="C17" s="5" t="n"/>
+      <c r="D17" s="5" t="n"/>
+      <c r="E17" s="5" t="n"/>
+      <c r="F17" s="5" t="n"/>
+      <c r="G17" s="5" t="n"/>
+      <c r="H17" s="5" t="n"/>
+      <c r="I17" s="5" t="n"/>
+      <c r="J17" s="5" t="n"/>
+      <c r="K17" s="5" t="n"/>
+      <c r="L17" s="5" t="n"/>
+      <c r="M17" s="5" t="n"/>
+      <c r="N17" s="5" t="n"/>
+      <c r="O17" s="5" t="n"/>
+      <c r="P17" s="5" t="n"/>
+      <c r="Q17" s="5" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="n"/>
+      <c r="B18" s="5" t="n"/>
+      <c r="C18" s="5" t="n"/>
+      <c r="D18" s="5" t="n"/>
+      <c r="E18" s="5" t="n"/>
+      <c r="F18" s="5" t="n"/>
+      <c r="G18" s="5" t="n"/>
+      <c r="H18" s="5" t="n"/>
+      <c r="I18" s="5" t="n"/>
+      <c r="J18" s="5" t="n"/>
+      <c r="K18" s="5" t="n"/>
+      <c r="L18" s="5" t="n"/>
+      <c r="M18" s="5" t="n"/>
+      <c r="N18" s="5" t="n"/>
+      <c r="O18" s="5" t="n"/>
+      <c r="P18" s="5" t="n"/>
+      <c r="Q18" s="5" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="n"/>
+      <c r="B19" s="5" t="n"/>
+      <c r="C19" s="5" t="n"/>
+      <c r="D19" s="5" t="n"/>
+      <c r="E19" s="5" t="n"/>
+      <c r="F19" s="5" t="n"/>
+      <c r="G19" s="5" t="n"/>
+      <c r="H19" s="5" t="n"/>
+      <c r="I19" s="5" t="n"/>
+      <c r="J19" s="5" t="n"/>
+      <c r="K19" s="5" t="n"/>
+      <c r="L19" s="5" t="n"/>
+      <c r="M19" s="5" t="n"/>
+      <c r="N19" s="5" t="n"/>
+      <c r="O19" s="5" t="n"/>
+      <c r="P19" s="5" t="n"/>
+      <c r="Q19" s="5" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="n"/>
+      <c r="B20" s="5" t="n"/>
+      <c r="C20" s="5" t="n"/>
+      <c r="D20" s="5" t="n"/>
+      <c r="E20" s="5" t="n"/>
+      <c r="F20" s="5" t="n"/>
+      <c r="G20" s="5" t="n"/>
+      <c r="H20" s="5" t="n"/>
+      <c r="I20" s="5" t="n"/>
+      <c r="J20" s="5" t="n"/>
+      <c r="K20" s="5" t="n"/>
+      <c r="L20" s="5" t="n"/>
+      <c r="M20" s="5" t="n"/>
+      <c r="N20" s="5" t="n"/>
+      <c r="O20" s="5" t="n"/>
+      <c r="P20" s="5" t="n"/>
+      <c r="Q20" s="5" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="n"/>
+      <c r="B21" s="5" t="n"/>
+      <c r="C21" s="5" t="n"/>
+      <c r="D21" s="5" t="n"/>
+      <c r="E21" s="5" t="n"/>
+      <c r="F21" s="5" t="n"/>
+      <c r="G21" s="5" t="n"/>
+      <c r="H21" s="5" t="n"/>
+      <c r="I21" s="5" t="n"/>
+      <c r="J21" s="5" t="n"/>
+      <c r="K21" s="5" t="n"/>
+      <c r="L21" s="5" t="n"/>
+      <c r="M21" s="5" t="n"/>
+      <c r="N21" s="5" t="n"/>
+      <c r="O21" s="5" t="n"/>
+      <c r="P21" s="5" t="n"/>
+      <c r="Q21" s="5" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="n"/>
+      <c r="B22" s="5" t="n"/>
+      <c r="C22" s="5" t="n"/>
+      <c r="D22" s="5" t="n"/>
+      <c r="E22" s="5" t="n"/>
+      <c r="F22" s="5" t="n"/>
+      <c r="G22" s="5" t="n"/>
+      <c r="H22" s="5" t="n"/>
+      <c r="I22" s="5" t="n"/>
+      <c r="J22" s="5" t="n"/>
+      <c r="K22" s="5" t="n"/>
+      <c r="L22" s="5" t="n"/>
+      <c r="M22" s="5" t="n"/>
+      <c r="N22" s="5" t="n"/>
+      <c r="O22" s="5" t="n"/>
+      <c r="P22" s="5" t="n"/>
+      <c r="Q22" s="5" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="n"/>
+      <c r="B23" s="5" t="n"/>
+      <c r="C23" s="5" t="n"/>
+      <c r="D23" s="5" t="n"/>
+      <c r="E23" s="5" t="n"/>
+      <c r="F23" s="5" t="n"/>
+      <c r="G23" s="5" t="n"/>
+      <c r="H23" s="5" t="n"/>
+      <c r="I23" s="5" t="n"/>
+      <c r="J23" s="5" t="n"/>
+      <c r="K23" s="5" t="n"/>
+      <c r="L23" s="5" t="n"/>
+      <c r="M23" s="5" t="n"/>
+      <c r="N23" s="5" t="n"/>
+      <c r="O23" s="5" t="n"/>
+      <c r="P23" s="5" t="n"/>
+      <c r="Q23" s="5" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="n"/>
+      <c r="B24" s="5" t="n"/>
+      <c r="C24" s="5" t="n"/>
+      <c r="D24" s="5" t="n"/>
+      <c r="E24" s="5" t="n"/>
+      <c r="F24" s="5" t="n"/>
+      <c r="G24" s="5" t="n"/>
+      <c r="H24" s="5" t="n"/>
+      <c r="I24" s="5" t="n"/>
+      <c r="J24" s="5" t="n"/>
+      <c r="K24" s="5" t="n"/>
+      <c r="L24" s="5" t="n"/>
+      <c r="M24" s="5" t="n"/>
+      <c r="N24" s="5" t="n"/>
+      <c r="O24" s="5" t="n"/>
+      <c r="P24" s="5" t="n"/>
+      <c r="Q24" s="5" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="n"/>
+      <c r="B25" s="5" t="n"/>
+      <c r="C25" s="5" t="n"/>
+      <c r="D25" s="5" t="n"/>
+      <c r="E25" s="5" t="n"/>
+      <c r="F25" s="5" t="n"/>
+      <c r="G25" s="5" t="n"/>
+      <c r="H25" s="5" t="n"/>
+      <c r="I25" s="5" t="n"/>
+      <c r="J25" s="5" t="n"/>
+      <c r="K25" s="5" t="n"/>
+      <c r="L25" s="5" t="n"/>
+      <c r="M25" s="5" t="n"/>
+      <c r="N25" s="5" t="n"/>
+      <c r="O25" s="5" t="n"/>
+      <c r="P25" s="5" t="n"/>
+      <c r="Q25" s="5" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="n"/>
+      <c r="B26" s="5" t="n"/>
+      <c r="C26" s="5" t="n"/>
+      <c r="D26" s="5" t="n"/>
+      <c r="E26" s="5" t="n"/>
+      <c r="F26" s="5" t="n"/>
+      <c r="G26" s="5" t="n"/>
+      <c r="H26" s="5" t="n"/>
+      <c r="I26" s="5" t="n"/>
+      <c r="J26" s="5" t="n"/>
+      <c r="K26" s="5" t="n"/>
+      <c r="L26" s="5" t="n"/>
+      <c r="M26" s="5" t="n"/>
+      <c r="N26" s="5" t="n"/>
+      <c r="O26" s="5" t="n"/>
+      <c r="P26" s="5" t="n"/>
+      <c r="Q26" s="5" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="n"/>
+      <c r="B27" s="5" t="n"/>
+      <c r="C27" s="5" t="n"/>
+      <c r="D27" s="5" t="n"/>
+      <c r="E27" s="5" t="n"/>
+      <c r="F27" s="5" t="n"/>
+      <c r="G27" s="5" t="n"/>
+      <c r="H27" s="5" t="n"/>
+      <c r="I27" s="5" t="n"/>
+      <c r="J27" s="5" t="n"/>
+      <c r="K27" s="5" t="n"/>
+      <c r="L27" s="5" t="n"/>
+      <c r="M27" s="5" t="n"/>
+      <c r="N27" s="5" t="n"/>
+      <c r="O27" s="5" t="n"/>
+      <c r="P27" s="5" t="n"/>
+      <c r="Q27" s="5" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="n"/>
+      <c r="B28" s="5" t="n"/>
+      <c r="C28" s="5" t="n"/>
+      <c r="D28" s="5" t="n"/>
+      <c r="E28" s="5" t="n"/>
+      <c r="F28" s="5" t="n"/>
+      <c r="G28" s="5" t="n"/>
+      <c r="H28" s="5" t="n"/>
+      <c r="I28" s="5" t="n"/>
+      <c r="J28" s="5" t="n"/>
+      <c r="K28" s="5" t="n"/>
+      <c r="L28" s="5" t="n"/>
+      <c r="M28" s="5" t="n"/>
+      <c r="N28" s="5" t="n"/>
+      <c r="O28" s="5" t="n"/>
+      <c r="P28" s="5" t="n"/>
+      <c r="Q28" s="5" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="n"/>
+      <c r="B29" s="5" t="n"/>
+      <c r="C29" s="5" t="n"/>
+      <c r="D29" s="5" t="n"/>
+      <c r="E29" s="5" t="n"/>
+      <c r="F29" s="5" t="n"/>
+      <c r="G29" s="5" t="n"/>
+      <c r="H29" s="5" t="n"/>
+      <c r="I29" s="5" t="n"/>
+      <c r="J29" s="5" t="n"/>
+      <c r="K29" s="5" t="n"/>
+      <c r="L29" s="5" t="n"/>
+      <c r="M29" s="5" t="n"/>
+      <c r="N29" s="5" t="n"/>
+      <c r="O29" s="5" t="n"/>
+      <c r="P29" s="5" t="n"/>
+      <c r="Q29" s="5" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="n"/>
+      <c r="B30" s="5" t="n"/>
+      <c r="C30" s="5" t="n"/>
+      <c r="D30" s="5" t="n"/>
+      <c r="E30" s="5" t="n"/>
+      <c r="F30" s="5" t="n"/>
+      <c r="G30" s="5" t="n"/>
+      <c r="H30" s="5" t="n"/>
+      <c r="I30" s="5" t="n"/>
+      <c r="J30" s="5" t="n"/>
+      <c r="K30" s="5" t="n"/>
+      <c r="L30" s="5" t="n"/>
+      <c r="M30" s="5" t="n"/>
+      <c r="N30" s="5" t="n"/>
+      <c r="O30" s="5" t="n"/>
+      <c r="P30" s="5" t="n"/>
+      <c r="Q30" s="5" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="n"/>
+      <c r="B31" s="5" t="n"/>
+      <c r="C31" s="5" t="n"/>
+      <c r="D31" s="5" t="n"/>
+      <c r="E31" s="5" t="n"/>
+      <c r="F31" s="5" t="n"/>
+      <c r="G31" s="5" t="n"/>
+      <c r="H31" s="5" t="n"/>
+      <c r="I31" s="5" t="n"/>
+      <c r="J31" s="5" t="n"/>
+      <c r="K31" s="5" t="n"/>
+      <c r="L31" s="5" t="n"/>
+      <c r="M31" s="5" t="n"/>
+      <c r="N31" s="5" t="n"/>
+      <c r="O31" s="5" t="n"/>
+      <c r="P31" s="5" t="n"/>
+      <c r="Q31" s="5" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="n"/>
+      <c r="B32" s="5" t="n"/>
+      <c r="C32" s="5" t="n"/>
+      <c r="D32" s="5" t="n"/>
+      <c r="E32" s="5" t="n"/>
+      <c r="F32" s="5" t="n"/>
+      <c r="G32" s="5" t="n"/>
+      <c r="H32" s="5" t="n"/>
+      <c r="I32" s="5" t="n"/>
+      <c r="J32" s="5" t="n"/>
+      <c r="K32" s="5" t="n"/>
+      <c r="L32" s="5" t="n"/>
+      <c r="M32" s="5" t="n"/>
+      <c r="N32" s="5" t="n"/>
+      <c r="O32" s="5" t="n"/>
+      <c r="P32" s="5" t="n"/>
+      <c r="Q32" s="5" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="n"/>
+      <c r="B33" s="5" t="n"/>
+      <c r="C33" s="5" t="n"/>
+      <c r="D33" s="5" t="n"/>
+      <c r="E33" s="5" t="n"/>
+      <c r="F33" s="5" t="n"/>
+      <c r="G33" s="5" t="n"/>
+      <c r="H33" s="5" t="n"/>
+      <c r="I33" s="5" t="n"/>
+      <c r="J33" s="5" t="n"/>
+      <c r="K33" s="5" t="n"/>
+      <c r="L33" s="5" t="n"/>
+      <c r="M33" s="5" t="n"/>
+      <c r="N33" s="5" t="n"/>
+      <c r="O33" s="5" t="n"/>
+      <c r="P33" s="5" t="n"/>
+      <c r="Q33" s="5" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="n"/>
+      <c r="B34" s="5" t="n"/>
+      <c r="C34" s="5" t="n"/>
+      <c r="D34" s="5" t="n"/>
+      <c r="E34" s="5" t="n"/>
+      <c r="F34" s="5" t="n"/>
+      <c r="G34" s="5" t="n"/>
+      <c r="H34" s="5" t="n"/>
+      <c r="I34" s="5" t="n"/>
+      <c r="J34" s="5" t="n"/>
+      <c r="K34" s="5" t="n"/>
+      <c r="L34" s="5" t="n"/>
+      <c r="M34" s="5" t="n"/>
+      <c r="N34" s="5" t="n"/>
+      <c r="O34" s="5" t="n"/>
+      <c r="P34" s="5" t="n"/>
+      <c r="Q34" s="5" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="n"/>
+      <c r="B35" s="5" t="n"/>
+      <c r="C35" s="5" t="n"/>
+      <c r="D35" s="5" t="n"/>
+      <c r="E35" s="5" t="n"/>
+      <c r="F35" s="5" t="n"/>
+      <c r="G35" s="5" t="n"/>
+      <c r="H35" s="5" t="n"/>
+      <c r="I35" s="5" t="n"/>
+      <c r="J35" s="5" t="n"/>
+      <c r="K35" s="5" t="n"/>
+      <c r="L35" s="5" t="n"/>
+      <c r="M35" s="5" t="n"/>
+      <c r="N35" s="5" t="n"/>
+      <c r="O35" s="5" t="n"/>
+      <c r="P35" s="5" t="n"/>
+      <c r="Q35" s="5" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="n"/>
+      <c r="B36" s="5" t="n"/>
+      <c r="C36" s="5" t="n"/>
+      <c r="D36" s="5" t="n"/>
+      <c r="E36" s="5" t="n"/>
+      <c r="F36" s="5" t="n"/>
+      <c r="G36" s="5" t="n"/>
+      <c r="H36" s="5" t="n"/>
+      <c r="I36" s="5" t="n"/>
+      <c r="J36" s="5" t="n"/>
+      <c r="K36" s="5" t="n"/>
+      <c r="L36" s="5" t="n"/>
+      <c r="M36" s="5" t="n"/>
+      <c r="N36" s="5" t="n"/>
+      <c r="O36" s="5" t="n"/>
+      <c r="P36" s="5" t="n"/>
+      <c r="Q36" s="5" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="n"/>
+      <c r="B37" s="5" t="n"/>
+      <c r="C37" s="5" t="n"/>
+      <c r="D37" s="5" t="n"/>
+      <c r="E37" s="5" t="n"/>
+      <c r="F37" s="5" t="n"/>
+      <c r="G37" s="5" t="n"/>
+      <c r="H37" s="5" t="n"/>
+      <c r="I37" s="5" t="n"/>
+      <c r="J37" s="5" t="n"/>
+      <c r="K37" s="5" t="n"/>
+      <c r="L37" s="5" t="n"/>
+      <c r="M37" s="5" t="n"/>
+      <c r="N37" s="5" t="n"/>
+      <c r="O37" s="5" t="n"/>
+      <c r="P37" s="5" t="n"/>
+      <c r="Q37" s="5" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="n"/>
+      <c r="B38" s="5" t="n"/>
+      <c r="C38" s="5" t="n"/>
+      <c r="D38" s="5" t="n"/>
+      <c r="E38" s="5" t="n"/>
+      <c r="F38" s="5" t="n"/>
+      <c r="G38" s="5" t="n"/>
+      <c r="H38" s="5" t="n"/>
+      <c r="I38" s="5" t="n"/>
+      <c r="J38" s="5" t="n"/>
+      <c r="K38" s="5" t="n"/>
+      <c r="L38" s="5" t="n"/>
+      <c r="M38" s="5" t="n"/>
+      <c r="N38" s="5" t="n"/>
+      <c r="O38" s="5" t="n"/>
+      <c r="P38" s="5" t="n"/>
+      <c r="Q38" s="5" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="n"/>
+      <c r="B39" s="5" t="n"/>
+      <c r="C39" s="5" t="n"/>
+      <c r="D39" s="5" t="n"/>
+      <c r="E39" s="5" t="n"/>
+      <c r="F39" s="5" t="n"/>
+      <c r="G39" s="5" t="n"/>
+      <c r="H39" s="5" t="n"/>
+      <c r="I39" s="5" t="n"/>
+      <c r="J39" s="5" t="n"/>
+      <c r="K39" s="5" t="n"/>
+      <c r="L39" s="5" t="n"/>
+      <c r="M39" s="5" t="n"/>
+      <c r="N39" s="5" t="n"/>
+      <c r="O39" s="5" t="n"/>
+      <c r="P39" s="5" t="n"/>
+      <c r="Q39" s="5" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="n"/>
+      <c r="B40" s="5" t="n"/>
+      <c r="C40" s="5" t="n"/>
+      <c r="D40" s="5" t="n"/>
+      <c r="E40" s="5" t="n"/>
+      <c r="F40" s="5" t="n"/>
+      <c r="G40" s="5" t="n"/>
+      <c r="H40" s="5" t="n"/>
+      <c r="I40" s="5" t="n"/>
+      <c r="J40" s="5" t="n"/>
+      <c r="K40" s="5" t="n"/>
+      <c r="L40" s="5" t="n"/>
+      <c r="M40" s="5" t="n"/>
+      <c r="N40" s="5" t="n"/>
+      <c r="O40" s="5" t="n"/>
+      <c r="P40" s="5" t="n"/>
+      <c r="Q40" s="5" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="n"/>
+      <c r="B41" s="5" t="n"/>
+      <c r="C41" s="5" t="n"/>
+      <c r="D41" s="5" t="n"/>
+      <c r="E41" s="5" t="n"/>
+      <c r="F41" s="5" t="n"/>
+      <c r="G41" s="5" t="n"/>
+      <c r="H41" s="5" t="n"/>
+      <c r="I41" s="5" t="n"/>
+      <c r="J41" s="5" t="n"/>
+      <c r="K41" s="5" t="n"/>
+      <c r="L41" s="5" t="n"/>
+      <c r="M41" s="5" t="n"/>
+      <c r="N41" s="5" t="n"/>
+      <c r="O41" s="5" t="n"/>
+      <c r="P41" s="5" t="n"/>
+      <c r="Q41" s="5" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="n"/>
+      <c r="B42" s="5" t="n"/>
+      <c r="C42" s="5" t="n"/>
+      <c r="D42" s="5" t="n"/>
+      <c r="E42" s="5" t="n"/>
+      <c r="F42" s="5" t="n"/>
+      <c r="G42" s="5" t="n"/>
+      <c r="H42" s="5" t="n"/>
+      <c r="I42" s="5" t="n"/>
+      <c r="J42" s="5" t="n"/>
+      <c r="K42" s="5" t="n"/>
+      <c r="L42" s="5" t="n"/>
+      <c r="M42" s="5" t="n"/>
+      <c r="N42" s="5" t="n"/>
+      <c r="O42" s="5" t="n"/>
+      <c r="P42" s="5" t="n"/>
+      <c r="Q42" s="5" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="n"/>
+      <c r="B43" s="5" t="n"/>
+      <c r="C43" s="5" t="n"/>
+      <c r="D43" s="5" t="n"/>
+      <c r="E43" s="5" t="n"/>
+      <c r="F43" s="5" t="n"/>
+      <c r="G43" s="5" t="n"/>
+      <c r="H43" s="5" t="n"/>
+      <c r="I43" s="5" t="n"/>
+      <c r="J43" s="5" t="n"/>
+      <c r="K43" s="5" t="n"/>
+      <c r="L43" s="5" t="n"/>
+      <c r="M43" s="5" t="n"/>
+      <c r="N43" s="5" t="n"/>
+      <c r="O43" s="5" t="n"/>
+      <c r="P43" s="5" t="n"/>
+      <c r="Q43" s="5" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="n"/>
+      <c r="B44" s="5" t="n"/>
+      <c r="C44" s="5" t="n"/>
+      <c r="D44" s="5" t="n"/>
+      <c r="E44" s="5" t="n"/>
+      <c r="F44" s="5" t="n"/>
+      <c r="G44" s="5" t="n"/>
+      <c r="H44" s="5" t="n"/>
+      <c r="I44" s="5" t="n"/>
+      <c r="J44" s="5" t="n"/>
+      <c r="K44" s="5" t="n"/>
+      <c r="L44" s="5" t="n"/>
+      <c r="M44" s="5" t="n"/>
+      <c r="N44" s="5" t="n"/>
+      <c r="O44" s="5" t="n"/>
+      <c r="P44" s="5" t="n"/>
+      <c r="Q44" s="5" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="n"/>
+      <c r="B45" s="5" t="n"/>
+      <c r="C45" s="5" t="n"/>
+      <c r="D45" s="5" t="n"/>
+      <c r="E45" s="5" t="n"/>
+      <c r="F45" s="5" t="n"/>
+      <c r="G45" s="5" t="n"/>
+      <c r="H45" s="5" t="n"/>
+      <c r="I45" s="5" t="n"/>
+      <c r="J45" s="5" t="n"/>
+      <c r="K45" s="5" t="n"/>
+      <c r="L45" s="5" t="n"/>
+      <c r="M45" s="5" t="n"/>
+      <c r="N45" s="5" t="n"/>
+      <c r="O45" s="5" t="n"/>
+      <c r="P45" s="5" t="n"/>
+      <c r="Q45" s="5" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="n"/>
+      <c r="B46" s="5" t="n"/>
+      <c r="C46" s="5" t="n"/>
+      <c r="D46" s="5" t="n"/>
+      <c r="E46" s="5" t="n"/>
+      <c r="F46" s="5" t="n"/>
+      <c r="G46" s="5" t="n"/>
+      <c r="H46" s="5" t="n"/>
+      <c r="I46" s="5" t="n"/>
+      <c r="J46" s="5" t="n"/>
+      <c r="K46" s="5" t="n"/>
+      <c r="L46" s="5" t="n"/>
+      <c r="M46" s="5" t="n"/>
+      <c r="N46" s="5" t="n"/>
+      <c r="O46" s="5" t="n"/>
+      <c r="P46" s="5" t="n"/>
+      <c r="Q46" s="5" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="n"/>
+      <c r="B47" s="5" t="n"/>
+      <c r="C47" s="5" t="n"/>
+      <c r="D47" s="5" t="n"/>
+      <c r="E47" s="5" t="n"/>
+      <c r="F47" s="5" t="n"/>
+      <c r="G47" s="5" t="n"/>
+      <c r="H47" s="5" t="n"/>
+      <c r="I47" s="5" t="n"/>
+      <c r="J47" s="5" t="n"/>
+      <c r="K47" s="5" t="n"/>
+      <c r="L47" s="5" t="n"/>
+      <c r="M47" s="5" t="n"/>
+      <c r="N47" s="5" t="n"/>
+      <c r="O47" s="5" t="n"/>
+      <c r="P47" s="5" t="n"/>
+      <c r="Q47" s="5" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="n"/>
+      <c r="B48" s="5" t="n"/>
+      <c r="C48" s="5" t="n"/>
+      <c r="D48" s="5" t="n"/>
+      <c r="E48" s="5" t="n"/>
+      <c r="F48" s="5" t="n"/>
+      <c r="G48" s="5" t="n"/>
+      <c r="H48" s="5" t="n"/>
+      <c r="I48" s="5" t="n"/>
+      <c r="J48" s="5" t="n"/>
+      <c r="K48" s="5" t="n"/>
+      <c r="L48" s="5" t="n"/>
+      <c r="M48" s="5" t="n"/>
+      <c r="N48" s="5" t="n"/>
+      <c r="O48" s="5" t="n"/>
+      <c r="P48" s="5" t="n"/>
+      <c r="Q48" s="5" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="n"/>
+      <c r="B49" s="5" t="n"/>
+      <c r="C49" s="5" t="n"/>
+      <c r="D49" s="5" t="n"/>
+      <c r="E49" s="5" t="n"/>
+      <c r="F49" s="5" t="n"/>
+      <c r="G49" s="5" t="n"/>
+      <c r="H49" s="5" t="n"/>
+      <c r="I49" s="5" t="n"/>
+      <c r="J49" s="5" t="n"/>
+      <c r="K49" s="5" t="n"/>
+      <c r="L49" s="5" t="n"/>
+      <c r="M49" s="5" t="n"/>
+      <c r="N49" s="5" t="n"/>
+      <c r="O49" s="5" t="n"/>
+      <c r="P49" s="5" t="n"/>
+      <c r="Q49" s="5" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="n"/>
+      <c r="B50" s="5" t="n"/>
+      <c r="C50" s="5" t="n"/>
+      <c r="D50" s="5" t="n"/>
+      <c r="E50" s="5" t="n"/>
+      <c r="F50" s="5" t="n"/>
+      <c r="G50" s="5" t="n"/>
+      <c r="H50" s="5" t="n"/>
+      <c r="I50" s="5" t="n"/>
+      <c r="J50" s="5" t="n"/>
+      <c r="K50" s="5" t="n"/>
+      <c r="L50" s="5" t="n"/>
+      <c r="M50" s="5" t="n"/>
+      <c r="N50" s="5" t="n"/>
+      <c r="O50" s="5" t="n"/>
+      <c r="P50" s="5" t="n"/>
+      <c r="Q50" s="5" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="n"/>
+      <c r="B51" s="5" t="n"/>
+      <c r="C51" s="5" t="n"/>
+      <c r="D51" s="5" t="n"/>
+      <c r="E51" s="5" t="n"/>
+      <c r="F51" s="5" t="n"/>
+      <c r="G51" s="5" t="n"/>
+      <c r="H51" s="5" t="n"/>
+      <c r="I51" s="5" t="n"/>
+      <c r="J51" s="5" t="n"/>
+      <c r="K51" s="5" t="n"/>
+      <c r="L51" s="5" t="n"/>
+      <c r="M51" s="5" t="n"/>
+      <c r="N51" s="5" t="n"/>
+      <c r="O51" s="5" t="n"/>
+      <c r="P51" s="5" t="n"/>
+      <c r="Q51" s="5" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="n"/>
+      <c r="B52" s="5" t="n"/>
+      <c r="C52" s="5" t="n"/>
+      <c r="D52" s="5" t="n"/>
+      <c r="E52" s="5" t="n"/>
+      <c r="F52" s="5" t="n"/>
+      <c r="G52" s="5" t="n"/>
+      <c r="H52" s="5" t="n"/>
+      <c r="I52" s="5" t="n"/>
+      <c r="J52" s="5" t="n"/>
+      <c r="K52" s="5" t="n"/>
+      <c r="L52" s="5" t="n"/>
+      <c r="M52" s="5" t="n"/>
+      <c r="N52" s="5" t="n"/>
+      <c r="O52" s="5" t="n"/>
+      <c r="P52" s="5" t="n"/>
+      <c r="Q52" s="5" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="n"/>
+      <c r="B53" s="5" t="n"/>
+      <c r="C53" s="5" t="n"/>
+      <c r="D53" s="5" t="n"/>
+      <c r="E53" s="5" t="n"/>
+      <c r="F53" s="5" t="n"/>
+      <c r="G53" s="5" t="n"/>
+      <c r="H53" s="5" t="n"/>
+      <c r="I53" s="5" t="n"/>
+      <c r="J53" s="5" t="n"/>
+      <c r="K53" s="5" t="n"/>
+      <c r="L53" s="5" t="n"/>
+      <c r="M53" s="5" t="n"/>
+      <c r="N53" s="5" t="n"/>
+      <c r="O53" s="5" t="n"/>
+      <c r="P53" s="5" t="n"/>
+      <c r="Q53" s="5" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="n"/>
+      <c r="B54" s="5" t="n"/>
+      <c r="C54" s="5" t="n"/>
+      <c r="D54" s="5" t="n"/>
+      <c r="E54" s="5" t="n"/>
+      <c r="F54" s="5" t="n"/>
+      <c r="G54" s="5" t="n"/>
+      <c r="H54" s="5" t="n"/>
+      <c r="I54" s="5" t="n"/>
+      <c r="J54" s="5" t="n"/>
+      <c r="K54" s="5" t="n"/>
+      <c r="L54" s="5" t="n"/>
+      <c r="M54" s="5" t="n"/>
+      <c r="N54" s="5" t="n"/>
+      <c r="O54" s="5" t="n"/>
+      <c r="P54" s="5" t="n"/>
+      <c r="Q54" s="5" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="n"/>
+      <c r="B55" s="5" t="n"/>
+      <c r="C55" s="5" t="n"/>
+      <c r="D55" s="5" t="n"/>
+      <c r="E55" s="5" t="n"/>
+      <c r="F55" s="5" t="n"/>
+      <c r="G55" s="5" t="n"/>
+      <c r="H55" s="5" t="n"/>
+      <c r="I55" s="5" t="n"/>
+      <c r="J55" s="5" t="n"/>
+      <c r="K55" s="5" t="n"/>
+      <c r="L55" s="5" t="n"/>
+      <c r="M55" s="5" t="n"/>
+      <c r="N55" s="5" t="n"/>
+      <c r="O55" s="5" t="n"/>
+      <c r="P55" s="5" t="n"/>
+      <c r="Q55" s="5" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="n"/>
+      <c r="B56" s="5" t="n"/>
+      <c r="C56" s="5" t="n"/>
+      <c r="D56" s="5" t="n"/>
+      <c r="E56" s="5" t="n"/>
+      <c r="F56" s="5" t="n"/>
+      <c r="G56" s="5" t="n"/>
+      <c r="H56" s="5" t="n"/>
+      <c r="I56" s="5" t="n"/>
+      <c r="J56" s="5" t="n"/>
+      <c r="K56" s="5" t="n"/>
+      <c r="L56" s="5" t="n"/>
+      <c r="M56" s="5" t="n"/>
+      <c r="N56" s="5" t="n"/>
+      <c r="O56" s="5" t="n"/>
+      <c r="P56" s="5" t="n"/>
+      <c r="Q56" s="5" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="n"/>
+      <c r="B57" s="5" t="n"/>
+      <c r="C57" s="5" t="n"/>
+      <c r="D57" s="5" t="n"/>
+      <c r="E57" s="5" t="n"/>
+      <c r="F57" s="5" t="n"/>
+      <c r="G57" s="5" t="n"/>
+      <c r="H57" s="5" t="n"/>
+      <c r="I57" s="5" t="n"/>
+      <c r="J57" s="5" t="n"/>
+      <c r="K57" s="5" t="n"/>
+      <c r="L57" s="5" t="n"/>
+      <c r="M57" s="5" t="n"/>
+      <c r="N57" s="5" t="n"/>
+      <c r="O57" s="5" t="n"/>
+      <c r="P57" s="5" t="n"/>
+      <c r="Q57" s="5" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="n"/>
+      <c r="B58" s="5" t="n"/>
+      <c r="C58" s="5" t="n"/>
+      <c r="D58" s="5" t="n"/>
+      <c r="E58" s="5" t="n"/>
+      <c r="F58" s="5" t="n"/>
+      <c r="G58" s="5" t="n"/>
+      <c r="H58" s="5" t="n"/>
+      <c r="I58" s="5" t="n"/>
+      <c r="J58" s="5" t="n"/>
+      <c r="K58" s="5" t="n"/>
+      <c r="L58" s="5" t="n"/>
+      <c r="M58" s="5" t="n"/>
+      <c r="N58" s="5" t="n"/>
+      <c r="O58" s="5" t="n"/>
+      <c r="P58" s="5" t="n"/>
+      <c r="Q58" s="5" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="5" t="n"/>
+      <c r="B59" s="5" t="n"/>
+      <c r="C59" s="5" t="n"/>
+      <c r="D59" s="5" t="n"/>
+      <c r="E59" s="5" t="n"/>
+      <c r="F59" s="5" t="n"/>
+      <c r="G59" s="5" t="n"/>
+      <c r="H59" s="5" t="n"/>
+      <c r="I59" s="5" t="n"/>
+      <c r="J59" s="5" t="n"/>
+      <c r="K59" s="5" t="n"/>
+      <c r="L59" s="5" t="n"/>
+      <c r="M59" s="5" t="n"/>
+      <c r="N59" s="5" t="n"/>
+      <c r="O59" s="5" t="n"/>
+      <c r="P59" s="5" t="n"/>
+      <c r="Q59" s="5" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="5" t="n"/>
+      <c r="B60" s="5" t="n"/>
+      <c r="C60" s="5" t="n"/>
+      <c r="D60" s="5" t="n"/>
+      <c r="E60" s="5" t="n"/>
+      <c r="F60" s="5" t="n"/>
+      <c r="G60" s="5" t="n"/>
+      <c r="H60" s="5" t="n"/>
+      <c r="I60" s="5" t="n"/>
+      <c r="J60" s="5" t="n"/>
+      <c r="K60" s="5" t="n"/>
+      <c r="L60" s="5" t="n"/>
+      <c r="M60" s="5" t="n"/>
+      <c r="N60" s="5" t="n"/>
+      <c r="O60" s="5" t="n"/>
+      <c r="P60" s="5" t="n"/>
+      <c r="Q60" s="5" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="5" t="n"/>
+      <c r="B61" s="5" t="n"/>
+      <c r="C61" s="5" t="n"/>
+      <c r="D61" s="5" t="n"/>
+      <c r="E61" s="5" t="n"/>
+      <c r="F61" s="5" t="n"/>
+      <c r="G61" s="5" t="n"/>
+      <c r="H61" s="5" t="n"/>
+      <c r="I61" s="5" t="n"/>
+      <c r="J61" s="5" t="n"/>
+      <c r="K61" s="5" t="n"/>
+      <c r="L61" s="5" t="n"/>
+      <c r="M61" s="5" t="n"/>
+      <c r="N61" s="5" t="n"/>
+      <c r="O61" s="5" t="n"/>
+      <c r="P61" s="5" t="n"/>
+      <c r="Q61" s="5" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="5" t="n"/>
+      <c r="B62" s="5" t="n"/>
+      <c r="C62" s="5" t="n"/>
+      <c r="D62" s="5" t="n"/>
+      <c r="E62" s="5" t="n"/>
+      <c r="F62" s="5" t="n"/>
+      <c r="G62" s="5" t="n"/>
+      <c r="H62" s="5" t="n"/>
+      <c r="I62" s="5" t="n"/>
+      <c r="J62" s="5" t="n"/>
+      <c r="K62" s="5" t="n"/>
+      <c r="L62" s="5" t="n"/>
+      <c r="M62" s="5" t="n"/>
+      <c r="N62" s="5" t="n"/>
+      <c r="O62" s="5" t="n"/>
+      <c r="P62" s="5" t="n"/>
+      <c r="Q62" s="5" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="5" t="n"/>
+      <c r="B63" s="5" t="n"/>
+      <c r="C63" s="5" t="n"/>
+      <c r="D63" s="5" t="n"/>
+      <c r="E63" s="5" t="n"/>
+      <c r="F63" s="5" t="n"/>
+      <c r="G63" s="5" t="n"/>
+      <c r="H63" s="5" t="n"/>
+      <c r="I63" s="5" t="n"/>
+      <c r="J63" s="5" t="n"/>
+      <c r="K63" s="5" t="n"/>
+      <c r="L63" s="5" t="n"/>
+      <c r="M63" s="5" t="n"/>
+      <c r="N63" s="5" t="n"/>
+      <c r="O63" s="5" t="n"/>
+      <c r="P63" s="5" t="n"/>
+      <c r="Q63" s="5" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="5" t="n"/>
+      <c r="B64" s="5" t="n"/>
+      <c r="C64" s="5" t="n"/>
+      <c r="D64" s="5" t="n"/>
+      <c r="E64" s="5" t="n"/>
+      <c r="F64" s="5" t="n"/>
+      <c r="G64" s="5" t="n"/>
+      <c r="H64" s="5" t="n"/>
+      <c r="I64" s="5" t="n"/>
+      <c r="J64" s="5" t="n"/>
+      <c r="K64" s="5" t="n"/>
+      <c r="L64" s="5" t="n"/>
+      <c r="M64" s="5" t="n"/>
+      <c r="N64" s="5" t="n"/>
+      <c r="O64" s="5" t="n"/>
+      <c r="P64" s="5" t="n"/>
+      <c r="Q64" s="5" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="5" t="n"/>
+      <c r="B65" s="5" t="n"/>
+      <c r="C65" s="5" t="n"/>
+      <c r="D65" s="5" t="n"/>
+      <c r="E65" s="5" t="n"/>
+      <c r="F65" s="5" t="n"/>
+      <c r="G65" s="5" t="n"/>
+      <c r="H65" s="5" t="n"/>
+      <c r="I65" s="5" t="n"/>
+      <c r="J65" s="5" t="n"/>
+      <c r="K65" s="5" t="n"/>
+      <c r="L65" s="5" t="n"/>
+      <c r="M65" s="5" t="n"/>
+      <c r="N65" s="5" t="n"/>
+      <c r="O65" s="5" t="n"/>
+      <c r="P65" s="5" t="n"/>
+      <c r="Q65" s="5" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="5" t="n"/>
+      <c r="B66" s="5" t="n"/>
+      <c r="C66" s="5" t="n"/>
+      <c r="D66" s="5" t="n"/>
+      <c r="E66" s="5" t="n"/>
+      <c r="F66" s="5" t="n"/>
+      <c r="G66" s="5" t="n"/>
+      <c r="H66" s="5" t="n"/>
+      <c r="I66" s="5" t="n"/>
+      <c r="J66" s="5" t="n"/>
+      <c r="K66" s="5" t="n"/>
+      <c r="L66" s="5" t="n"/>
+      <c r="M66" s="5" t="n"/>
+      <c r="N66" s="5" t="n"/>
+      <c r="O66" s="5" t="n"/>
+      <c r="P66" s="5" t="n"/>
+      <c r="Q66" s="5" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="5" t="n"/>
+      <c r="B67" s="5" t="n"/>
+      <c r="C67" s="5" t="n"/>
+      <c r="D67" s="5" t="n"/>
+      <c r="E67" s="5" t="n"/>
+      <c r="F67" s="5" t="n"/>
+      <c r="G67" s="5" t="n"/>
+      <c r="H67" s="5" t="n"/>
+      <c r="I67" s="5" t="n"/>
+      <c r="J67" s="5" t="n"/>
+      <c r="K67" s="5" t="n"/>
+      <c r="L67" s="5" t="n"/>
+      <c r="M67" s="5" t="n"/>
+      <c r="N67" s="5" t="n"/>
+      <c r="O67" s="5" t="n"/>
+      <c r="P67" s="5" t="n"/>
+      <c r="Q67" s="5" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="5" t="n"/>
+      <c r="B68" s="5" t="n"/>
+      <c r="C68" s="5" t="n"/>
+      <c r="D68" s="5" t="n"/>
+      <c r="E68" s="5" t="n"/>
+      <c r="F68" s="5" t="n"/>
+      <c r="G68" s="5" t="n"/>
+      <c r="H68" s="5" t="n"/>
+      <c r="I68" s="5" t="n"/>
+      <c r="J68" s="5" t="n"/>
+      <c r="K68" s="5" t="n"/>
+      <c r="L68" s="5" t="n"/>
+      <c r="M68" s="5" t="n"/>
+      <c r="N68" s="5" t="n"/>
+      <c r="O68" s="5" t="n"/>
+      <c r="P68" s="5" t="n"/>
+      <c r="Q68" s="5" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="5" t="n"/>
+      <c r="B69" s="5" t="n"/>
+      <c r="C69" s="5" t="n"/>
+      <c r="D69" s="5" t="n"/>
+      <c r="E69" s="5" t="n"/>
+      <c r="F69" s="5" t="n"/>
+      <c r="G69" s="5" t="n"/>
+      <c r="H69" s="5" t="n"/>
+      <c r="I69" s="5" t="n"/>
+      <c r="J69" s="5" t="n"/>
+      <c r="K69" s="5" t="n"/>
+      <c r="L69" s="5" t="n"/>
+      <c r="M69" s="5" t="n"/>
+      <c r="N69" s="5" t="n"/>
+      <c r="O69" s="5" t="n"/>
+      <c r="P69" s="5" t="n"/>
+      <c r="Q69" s="5" t="n"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="5" t="n"/>
+      <c r="B70" s="5" t="n"/>
+      <c r="C70" s="5" t="n"/>
+      <c r="D70" s="5" t="n"/>
+      <c r="E70" s="5" t="n"/>
+      <c r="F70" s="5" t="n"/>
+      <c r="G70" s="5" t="n"/>
+      <c r="H70" s="5" t="n"/>
+      <c r="I70" s="5" t="n"/>
+      <c r="J70" s="5" t="n"/>
+      <c r="K70" s="5" t="n"/>
+      <c r="L70" s="5" t="n"/>
+      <c r="M70" s="5" t="n"/>
+      <c r="N70" s="5" t="n"/>
+      <c r="O70" s="5" t="n"/>
+      <c r="P70" s="5" t="n"/>
+      <c r="Q70" s="5" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="5" t="n"/>
+      <c r="B71" s="5" t="n"/>
+      <c r="C71" s="5" t="n"/>
+      <c r="D71" s="5" t="n"/>
+      <c r="E71" s="5" t="n"/>
+      <c r="F71" s="5" t="n"/>
+      <c r="G71" s="5" t="n"/>
+      <c r="H71" s="5" t="n"/>
+      <c r="I71" s="5" t="n"/>
+      <c r="J71" s="5" t="n"/>
+      <c r="K71" s="5" t="n"/>
+      <c r="L71" s="5" t="n"/>
+      <c r="M71" s="5" t="n"/>
+      <c r="N71" s="5" t="n"/>
+      <c r="O71" s="5" t="n"/>
+      <c r="P71" s="5" t="n"/>
+      <c r="Q71" s="5" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="5" t="n"/>
+      <c r="B72" s="5" t="n"/>
+      <c r="C72" s="5" t="n"/>
+      <c r="D72" s="5" t="n"/>
+      <c r="E72" s="5" t="n"/>
+      <c r="F72" s="5" t="n"/>
+      <c r="G72" s="5" t="n"/>
+      <c r="H72" s="5" t="n"/>
+      <c r="I72" s="5" t="n"/>
+      <c r="J72" s="5" t="n"/>
+      <c r="K72" s="5" t="n"/>
+      <c r="L72" s="5" t="n"/>
+      <c r="M72" s="5" t="n"/>
+      <c r="N72" s="5" t="n"/>
+      <c r="O72" s="5" t="n"/>
+      <c r="P72" s="5" t="n"/>
+      <c r="Q72" s="5" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="5" t="n"/>
+      <c r="B73" s="5" t="n"/>
+      <c r="C73" s="5" t="n"/>
+      <c r="D73" s="5" t="n"/>
+      <c r="E73" s="5" t="n"/>
+      <c r="F73" s="5" t="n"/>
+      <c r="G73" s="5" t="n"/>
+      <c r="H73" s="5" t="n"/>
+      <c r="I73" s="5" t="n"/>
+      <c r="J73" s="5" t="n"/>
+      <c r="K73" s="5" t="n"/>
+      <c r="L73" s="5" t="n"/>
+      <c r="M73" s="5" t="n"/>
+      <c r="N73" s="5" t="n"/>
+      <c r="O73" s="5" t="n"/>
+      <c r="P73" s="5" t="n"/>
+      <c r="Q73" s="5" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="5" t="n"/>
+      <c r="B74" s="5" t="n"/>
+      <c r="C74" s="5" t="n"/>
+      <c r="D74" s="5" t="n"/>
+      <c r="E74" s="5" t="n"/>
+      <c r="F74" s="5" t="n"/>
+      <c r="G74" s="5" t="n"/>
+      <c r="H74" s="5" t="n"/>
+      <c r="I74" s="5" t="n"/>
+      <c r="J74" s="5" t="n"/>
+      <c r="K74" s="5" t="n"/>
+      <c r="L74" s="5" t="n"/>
+      <c r="M74" s="5" t="n"/>
+      <c r="N74" s="5" t="n"/>
+      <c r="O74" s="5" t="n"/>
+      <c r="P74" s="5" t="n"/>
+      <c r="Q74" s="5" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="5" t="n"/>
+      <c r="B75" s="5" t="n"/>
+      <c r="C75" s="5" t="n"/>
+      <c r="D75" s="5" t="n"/>
+      <c r="E75" s="5" t="n"/>
+      <c r="F75" s="5" t="n"/>
+      <c r="G75" s="5" t="n"/>
+      <c r="H75" s="5" t="n"/>
+      <c r="I75" s="5" t="n"/>
+      <c r="J75" s="5" t="n"/>
+      <c r="K75" s="5" t="n"/>
+      <c r="L75" s="5" t="n"/>
+      <c r="M75" s="5" t="n"/>
+      <c r="N75" s="5" t="n"/>
+      <c r="O75" s="5" t="n"/>
+      <c r="P75" s="5" t="n"/>
+      <c r="Q75" s="5" t="n"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="5" t="n"/>
+      <c r="B76" s="5" t="n"/>
+      <c r="C76" s="5" t="n"/>
+      <c r="D76" s="5" t="n"/>
+      <c r="E76" s="5" t="n"/>
+      <c r="F76" s="5" t="n"/>
+      <c r="G76" s="5" t="n"/>
+      <c r="H76" s="5" t="n"/>
+      <c r="I76" s="5" t="n"/>
+      <c r="J76" s="5" t="n"/>
+      <c r="K76" s="5" t="n"/>
+      <c r="L76" s="5" t="n"/>
+      <c r="M76" s="5" t="n"/>
+      <c r="N76" s="5" t="n"/>
+      <c r="O76" s="5" t="n"/>
+      <c r="P76" s="5" t="n"/>
+      <c r="Q76" s="5" t="n"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="5" t="n"/>
+      <c r="B77" s="5" t="n"/>
+      <c r="C77" s="5" t="n"/>
+      <c r="D77" s="5" t="n"/>
+      <c r="E77" s="5" t="n"/>
+      <c r="F77" s="5" t="n"/>
+      <c r="G77" s="5" t="n"/>
+      <c r="H77" s="5" t="n"/>
+      <c r="I77" s="5" t="n"/>
+      <c r="J77" s="5" t="n"/>
+      <c r="K77" s="5" t="n"/>
+      <c r="L77" s="5" t="n"/>
+      <c r="M77" s="5" t="n"/>
+      <c r="N77" s="5" t="n"/>
+      <c r="O77" s="5" t="n"/>
+      <c r="P77" s="5" t="n"/>
+      <c r="Q77" s="5" t="n"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="5" t="n"/>
+      <c r="B78" s="5" t="n"/>
+      <c r="C78" s="5" t="n"/>
+      <c r="D78" s="5" t="n"/>
+      <c r="E78" s="5" t="n"/>
+      <c r="F78" s="5" t="n"/>
+      <c r="G78" s="5" t="n"/>
+      <c r="H78" s="5" t="n"/>
+      <c r="I78" s="5" t="n"/>
+      <c r="J78" s="5" t="n"/>
+      <c r="K78" s="5" t="n"/>
+      <c r="L78" s="5" t="n"/>
+      <c r="M78" s="5" t="n"/>
+      <c r="N78" s="5" t="n"/>
+      <c r="O78" s="5" t="n"/>
+      <c r="P78" s="5" t="n"/>
+      <c r="Q78" s="5" t="n"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="5" t="n"/>
+      <c r="B79" s="5" t="n"/>
+      <c r="C79" s="5" t="n"/>
+      <c r="D79" s="5" t="n"/>
+      <c r="E79" s="5" t="n"/>
+      <c r="F79" s="5" t="n"/>
+      <c r="G79" s="5" t="n"/>
+      <c r="H79" s="5" t="n"/>
+      <c r="I79" s="5" t="n"/>
+      <c r="J79" s="5" t="n"/>
+      <c r="K79" s="5" t="n"/>
+      <c r="L79" s="5" t="n"/>
+      <c r="M79" s="5" t="n"/>
+      <c r="N79" s="5" t="n"/>
+      <c r="O79" s="5" t="n"/>
+      <c r="P79" s="5" t="n"/>
+      <c r="Q79" s="5" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -724,37 +2274,37 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
+      <c r="A1" s="6" t="inlineStr">
         <is>
           <t>Muestra</t>
         </is>
       </c>
-      <c r="B1" s="5" t="inlineStr">
+      <c r="B1" s="6" t="inlineStr">
         <is>
           <t>Gen</t>
         </is>
       </c>
-      <c r="C1" s="5" t="inlineStr">
+      <c r="C1" s="6" t="inlineStr">
         <is>
           <t>Ct 1</t>
         </is>
       </c>
-      <c r="D1" s="5" t="inlineStr">
+      <c r="D1" s="6" t="inlineStr">
         <is>
           <t>Ct 2</t>
         </is>
       </c>
-      <c r="E1" s="5" t="inlineStr">
+      <c r="E1" s="6" t="inlineStr">
         <is>
           <t>Ct Mean</t>
         </is>
       </c>
-      <c r="F1" s="5" t="inlineStr">
+      <c r="F1" s="6" t="inlineStr">
         <is>
           <t>Ct SD</t>
         </is>
       </c>
-      <c r="G1" s="5" t="inlineStr">
+      <c r="G1" s="6" t="inlineStr">
         <is>
           <t>Indet</t>
         </is>
@@ -775,47 +2325,47 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
+      <c r="A1" s="6" t="inlineStr">
         <is>
           <t>Muestra</t>
         </is>
       </c>
-      <c r="B1" s="5" t="inlineStr">
+      <c r="B1" s="6" t="inlineStr">
         <is>
           <t>Ct GOI</t>
         </is>
       </c>
-      <c r="C1" s="5" t="inlineStr">
+      <c r="C1" s="6" t="inlineStr">
         <is>
           <t>Ct PPIA</t>
         </is>
       </c>
-      <c r="D1" s="5" t="inlineStr">
+      <c r="D1" s="6" t="inlineStr">
         <is>
           <t>Ct SYP</t>
         </is>
       </c>
-      <c r="E1" s="5" t="inlineStr">
+      <c r="E1" s="6" t="inlineStr">
         <is>
           <t>dCt PPIA</t>
         </is>
       </c>
-      <c r="F1" s="5" t="inlineStr">
+      <c r="F1" s="6" t="inlineStr">
         <is>
           <t>dCt SYP</t>
         </is>
       </c>
-      <c r="G1" s="5" t="inlineStr">
+      <c r="G1" s="6" t="inlineStr">
         <is>
           <t>Gen interes</t>
         </is>
       </c>
-      <c r="H1" s="5" t="inlineStr">
+      <c r="H1" s="6" t="inlineStr">
         <is>
           <t>Prom dCt (C) PPIA</t>
         </is>
       </c>
-      <c r="I1" s="5" t="inlineStr">
+      <c r="I1" s="6" t="inlineStr">
         <is>
           <t>Prom dCt (C) SYP</t>
         </is>
@@ -824,4 +2374,18 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
qPCR 4.3.1: quitar hebras ADN de las hojas y no duplicar banner RAW; colores GLOBAL
- Las hebras de ADN solo van en el banner de la cabecera de RAW (incluido en la
  plantilla). La macro ya NO añade su propio banner -> no se duplica.
- Quitada la decoracion de esquina ADN en Instrucciones/Resultados/GLOBAL/Datos/
  Calculos (molestaba y quedaba mal).
- DecorarHojasLab -> LimpiarDecoracionHojas: solo elimina decoraciones antiguas,
  ya no pinta la fila 1 de teal. Asi GLOBAL recupera amarillo (controles) y verde
  (grupos), y Resultados sus colores.
- Eliminado dna_esquina.png y su generacion; generar_assets_lab.py solo crea el
  banner de RAW.
- Plantilla regenerada; version macro 4.3 -> 4.3.1. Calculo/deteccion SIN cambios.

Co-authored-by: carlosvibecoding <carlosvibecoding@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/qPCR_plantilla.xlsx
+++ b/qPCR_plantilla.xlsx
@@ -116,7 +116,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -147,7 +147,6 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -229,36 +228,6 @@
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>3</col>
-      <colOff>0</colOff>
-      <row>0</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="285750" cy="285750"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="1" name="Image 1" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-</wsDr>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <oneCellAnchor>
-    <from>
       <col>0</col>
       <colOff>0</colOff>
       <row>0</row>
@@ -285,127 +254,7 @@
 </wsDr>
 </file>
 
-<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <oneCellAnchor>
-    <from>
-      <col>7</col>
-      <colOff>0</colOff>
-      <row>0</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="285750" cy="285750"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="1" name="Image 1" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-</wsDr>
-</file>
-
-<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <oneCellAnchor>
-    <from>
-      <col>7</col>
-      <colOff>0</colOff>
-      <row>0</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="285750" cy="285750"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="1" name="Image 1" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-</wsDr>
-</file>
-
-<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <oneCellAnchor>
-    <from>
-      <col>7</col>
-      <colOff>0</colOff>
-      <row>0</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="285750" cy="285750"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="1" name="Image 1" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-</wsDr>
-</file>
-
-<file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <oneCellAnchor>
-    <from>
-      <col>7</col>
-      <colOff>0</colOff>
-      <row>0</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="285750" cy="285750"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="1" name="Image 1" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-</wsDr>
-</file>
-
-<file path=xl/drawings/drawing7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
@@ -447,31 +296,6 @@
       </nvPicPr>
       <blipFill>
         <a:blip cstate="print" r:embed="rId2"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>15</col>
-      <colOff>0</colOff>
-      <row>0</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="285750" cy="285750"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="3" name="Image 3" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId3"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -774,7 +598,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D27"/>
+  <dimension ref="A1:B27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="95" customWidth="1" min="1" max="1"/>
@@ -788,8 +612,6 @@
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr"/>
@@ -936,7 +758,7 @@
       </c>
       <c r="B23" s="9" t="inlineStr">
         <is>
-          <t>Clic en el raton (columna O, hoja RAW) = Procesar placa (macro 4.3)</t>
+          <t>Clic en el raton (columna O, hoja RAW) = Procesar placa (macro 4.3.1)</t>
         </is>
       </c>
     </row>
@@ -970,7 +792,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2341,22 +2162,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:A1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" ht="18" customHeight="1">
-      <c r="A1" s="2" t="n"/>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="2" t="n"/>
-    </row>
-  </sheetData>
+  <sheetData/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2366,22 +2175,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:A1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" ht="18" customHeight="1">
-      <c r="A1" s="2" t="n"/>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="2" t="n"/>
-    </row>
-  </sheetData>
+  <sheetData/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2391,10 +2188,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:G1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" ht="18" customHeight="1">
+    <row r="1">
       <c r="A1" s="16" t="inlineStr">
         <is>
           <t>Muestra</t>
@@ -2430,11 +2227,9 @@
           <t>Indet</t>
         </is>
       </c>
-      <c r="H1" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2447,7 +2242,7 @@
   <dimension ref="A1:I1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" ht="18" customHeight="1">
+    <row r="1">
       <c r="A1" s="16" t="inlineStr">
         <is>
           <t>Muestra</t>
@@ -2488,7 +2283,7 @@
           <t>Prom dCt (C) PPIA</t>
         </is>
       </c>
-      <c r="I1" s="17" t="inlineStr">
+      <c r="I1" s="16" t="inlineStr">
         <is>
           <t>Prom dCt (C) SYP</t>
         </is>
@@ -2496,7 +2291,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2512,7 +2306,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Recursos gráficos qPCR (no borrar). Orden: 1 raton, 2 banner, 3 esquina.</t>
+          <t>Recursos gráficos qPCR (no borrar). Orden: 1 raton, 2 banner.</t>
         </is>
       </c>
     </row>

</xml_diff>